<commit_message>
base: création de l'accueil & ajustement du nommage des URL, nom de route, contrôleur, gabarit Twig conformément au Schéma ergonomique
</commit_message>
<xml_diff>
--- a/documents/conceptualisation/specifications/Specifications.xlsx
+++ b/documents/conceptualisation/specifications/Specifications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell Pro\Desktop\EXAMEN_2026\FRAMEWORK_ADELINE-SIVAZ_2026\voisin-adeline\documents\conceptualisation\specifications\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47D9AEA2-DF9E-4832-B971-A23F7AFB66A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7A5B4F9-8BD4-4A50-B454-D6A90EB8802B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="-16200" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -198,7 +198,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>Déconnexion</t>
+      <t>Fil d'actualité membre</t>
     </r>
     <r>
       <rPr>
@@ -217,7 +217,151 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> Déconnecte l'utilisateur, repasse </t>
+      <t xml:space="preserve"> Affiche toutes les publications publiques et privées des amis. Gère le formulaire de création de post lié au connecté avec date automatique. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Gère le filtre GET (Tout, public, privé)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mes publications</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Affiche uniquement les publications écrites par l'utilisateur connecté.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Publications des amis</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Affiche uniquement les publications des membres présents dans la liste d'amis.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Détail d'une publication</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Affiche l'article complet, son nombre total de likes et la liste complète de ses commentaires associés.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Modification publication</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Affiche le formulaire. Enregistre les changements et la </t>
     </r>
     <r>
       <rPr>
@@ -226,17 +370,99 @@
         <rFont val="Courier New"/>
         <family val="3"/>
       </rPr>
-      <t>est_en_ligne</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> à </t>
+      <t>date_modification</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> automatique. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Sécurité :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Vérifie que le connecté est l'auteur.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Suppression publication</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Supprime définitivement la publication si l'utilisateur en est l'auteur. Gère les messages d'erreur.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Profil d'un membre </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Affiche les infos, la date d'inscription et la liste d'amis. Affiche les posts du membre selon le registre </t>
     </r>
     <r>
       <rPr>
@@ -245,29 +471,29 @@
         <rFont val="Courier New"/>
         <family val="3"/>
       </rPr>
-      <t>faux</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> et redirige vers l'accueil public.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Fil d'actualité membre</t>
+      <t>AutorisationAmi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Modification Profil</t>
     </r>
     <r>
       <rPr>
@@ -286,39 +512,19 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> Affiche toutes les publications publiques et privées des amis. Gère le formulaire de création de post lié au connecté avec date automatique. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Gère le filtre GET (Tout, public, privé)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Mes publications</t>
+      <t xml:space="preserve"> Formulaire de modification de la biographie ou de la photo de profil. Enregistre les changements avec messages d'erreur.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Créer un commentaire</t>
     </r>
     <r>
       <rPr>
@@ -337,100 +543,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> Affiche uniquement les publications écrites par l'utilisateur connecté.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Publications des amis</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Affiche uniquement les publications des membres présents dans la liste d'amis.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Détail d'une publication</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Affiche l'article complet, son nombre total de likes et la liste complète de ses commentaires associés.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Modification publication</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Affiche le formulaire. Enregistre les changements et la </t>
+      <t xml:space="preserve"> Enregistre un message sous un post, l'associe au connecté, génère automatiquement la </t>
     </r>
     <r>
       <rPr>
@@ -439,49 +552,60 @@
         <rFont val="Courier New"/>
         <family val="3"/>
       </rPr>
-      <t>date_modification</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> automatique. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Sécurité :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Vérifie que le connecté est l'auteur.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Suppression publication</t>
+      <t>date_creation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Gère les erreurs.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Modifier un commentaire </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Enregistre la modification du texte si le connecté en est l'auteur. Gère les erreurs.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mes demandes</t>
     </r>
     <r>
       <rPr>
@@ -500,38 +624,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> Supprime définitivement la publication si l'utilisateur en est l'auteur. Gère les messages d'erreur.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Profil d'un membre </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Affiche les infos, la date d'inscription et la liste d'amis. Affiche les posts du membre selon le registre </t>
+      <t xml:space="preserve"> Affiche la liste complète des demandes d'amitié reçues au statut </t>
     </r>
     <r>
       <rPr>
@@ -540,7 +633,7 @@
         <rFont val="Courier New"/>
         <family val="3"/>
       </rPr>
-      <t>AutorisationAmi</t>
+      <t>'en attente'</t>
     </r>
     <r>
       <rPr>
@@ -562,57 +655,26 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>Modification Profil</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Formulaire de modification de la biographie ou de la photo de profil. Enregistre les changements avec messages d'erreur.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Créer un commentaire</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Enregistre un message sous un post, l'associe au connecté, génère automatiquement la </t>
+      <t xml:space="preserve">Envoyer une demande </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Enregistre une nouvelle ligne dans </t>
     </r>
     <r>
       <rPr>
@@ -621,79 +683,17 @@
         <rFont val="Courier New"/>
         <family val="3"/>
       </rPr>
-      <t>date_creation</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. Gère les erreurs.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Modifier un commentaire </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Enregistre la modification du texte si le connecté en est l'auteur. Gère les erreurs.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Mes demandes</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Affiche la liste complète des demandes d'amitié reçues au statut </t>
+      <t>DemandeAmi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> au statut </t>
     </r>
     <r>
       <rPr>
@@ -712,38 +712,67 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Envoyer une demande </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Enregistre une nouvelle ligne dans </t>
+      <t xml:space="preserve"> avec la date du jour.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Supprimer un commentaire</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Supprime le commentaire si le connecté en est l'auteur.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Liste d'amis</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Parcourt le registre </t>
     </r>
     <r>
       <rPr>
@@ -752,17 +781,35 @@
         <rFont val="Courier New"/>
         <family val="3"/>
       </rPr>
-      <t>DemandeAmi</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> au statut </t>
+      <t>AutorisationAmi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>pour afficher tous les amis du connecté et met en avant ceux dont</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
@@ -771,77 +818,35 @@
         <rFont val="Courier New"/>
         <family val="3"/>
       </rPr>
-      <t>'en attente'</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> avec la date du jour.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Supprimer un commentaire</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Supprime le commentaire si le connecté en est l'auteur.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Liste d'amis</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Parcourt le registre </t>
+      <t>est_en_ligne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>est à</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
@@ -850,7 +855,7 @@
         <rFont val="Courier New"/>
         <family val="3"/>
       </rPr>
-      <t>AutorisationAmi</t>
+      <t>vrai</t>
     </r>
     <r>
       <rPr>
@@ -859,80 +864,6 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>pour afficher tous les amis du connecté et met en avant ceux dont</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Courier New"/>
-        <family val="3"/>
-      </rPr>
-      <t>est_en_ligne</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>est à</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Courier New"/>
-        <family val="3"/>
-      </rPr>
-      <t>vrai</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
       <t>.</t>
     </r>
   </si>
@@ -1025,9 +956,6 @@
   </si>
   <si>
     <t>security/connexion.html.twig</t>
-  </si>
-  <si>
-    <t>Redirection vers app_accueil_public</t>
   </si>
   <si>
     <t>SecurityController::deconnexion()</t>
@@ -1524,6 +1452,78 @@
   </si>
   <si>
     <t>app_demande_ami</t>
+  </si>
+  <si>
+    <t>Redirection → vers app_accueil_public</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Déconnexion</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Déconnecte l'utilisateur, repasse </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>est_en_ligne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> à </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>faux</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> et redirige → vers l'accueil public.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1984,13 +1984,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -2010,7 +2010,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>23</v>
@@ -2022,7 +2022,7 @@
         <v>6</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>14</v>
@@ -2036,19 +2036,19 @@
         <v>5</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>7</v>
@@ -2062,51 +2062,51 @@
         <v>5</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>71</v>
+        <v>133</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>26</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -2114,467 +2114,467 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>76</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>9</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>12</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>13</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>16</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>14</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D12" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>92</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>8</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G13" s="4" t="s">
         <v>8</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>8</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>20</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G15" s="4" t="s">
         <v>10</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G16" s="4" t="s">
         <v>10</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G17" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>10</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>21</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G19" s="4" t="s">
         <v>22</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="48" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>117</v>
-      </c>
       <c r="E20" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G20" s="4" t="s">
         <v>19</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>17</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G22" s="4" t="s">
         <v>18</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G23" s="4" t="s">
         <v>18</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>